<commit_message>
Fixed bugs and errors
</commit_message>
<xml_diff>
--- a/books_store/books_copy.xlsx
+++ b/books_store/books_copy.xlsx
@@ -569,7 +569,7 @@
         <v>75</v>
       </c>
       <c r="J2" s="3" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3">
@@ -611,7 +611,7 @@
         <v>105</v>
       </c>
       <c r="J3" s="3" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4">
@@ -653,7 +653,7 @@
         <v>87</v>
       </c>
       <c r="J4" s="3" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="5">
@@ -695,7 +695,7 @@
         <v>93</v>
       </c>
       <c r="J5" s="3" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="6">
@@ -737,7 +737,7 @@
         <v>82</v>
       </c>
       <c r="J6" s="3" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="7">
@@ -779,7 +779,7 @@
         <v>105</v>
       </c>
       <c r="J7" s="3" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="8">
@@ -821,7 +821,7 @@
         <v>120</v>
       </c>
       <c r="J8" s="3" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="9">
@@ -863,7 +863,7 @@
         <v>120</v>
       </c>
       <c r="J9" s="3" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="10">
@@ -905,7 +905,7 @@
         <v>105</v>
       </c>
       <c r="J10" s="3" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="11">
@@ -947,7 +947,7 @@
         <v>88</v>
       </c>
       <c r="J11" s="3" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -1066,7 +1066,7 @@
         <v>75</v>
       </c>
       <c r="J2" s="3" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="3">
@@ -1108,7 +1108,7 @@
         <v>120</v>
       </c>
       <c r="J3" s="3" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4">
@@ -1150,7 +1150,7 @@
         <v>90</v>
       </c>
       <c r="J4" s="3" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="5">
@@ -1192,7 +1192,7 @@
         <v>67</v>
       </c>
       <c r="J5" s="3" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="6">
@@ -1234,7 +1234,7 @@
         <v>60</v>
       </c>
       <c r="J6" s="3" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7">
@@ -1276,7 +1276,7 @@
         <v>90</v>
       </c>
       <c r="J7" s="3" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="8">
@@ -1318,7 +1318,7 @@
         <v>99</v>
       </c>
       <c r="J8" s="3" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="9">
@@ -1360,7 +1360,7 @@
         <v>75</v>
       </c>
       <c r="J9" s="3" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10">
@@ -1402,7 +1402,7 @@
         <v>90</v>
       </c>
       <c r="J10" s="3" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="11">
@@ -1444,7 +1444,7 @@
         <v>90</v>
       </c>
       <c r="J11" s="3" t="n">
-        <v>321</v>
+        <v>319</v>
       </c>
     </row>
   </sheetData>
@@ -1564,7 +1564,7 @@
         <v>90</v>
       </c>
       <c r="J2" s="3" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="3">
@@ -1606,7 +1606,7 @@
         <v>180</v>
       </c>
       <c r="J3" s="3" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4">
@@ -1648,7 +1648,7 @@
         <v>96</v>
       </c>
       <c r="J4" s="3" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="5">
@@ -1690,7 +1690,7 @@
         <v>105</v>
       </c>
       <c r="J5" s="3" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6">
@@ -1732,7 +1732,7 @@
         <v>90</v>
       </c>
       <c r="J6" s="3" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="7">
@@ -1774,7 +1774,7 @@
         <v>105</v>
       </c>
       <c r="J7" s="3" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="8">
@@ -1816,7 +1816,7 @@
         <v>120</v>
       </c>
       <c r="J8" s="3" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="9">
@@ -1858,7 +1858,7 @@
         <v>120</v>
       </c>
       <c r="J9" s="3" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="10">
@@ -1900,7 +1900,7 @@
         <v>75</v>
       </c>
       <c r="J10" s="3" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="11">
@@ -1942,7 +1942,7 @@
         <v>90</v>
       </c>
       <c r="J11" s="3" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -2061,7 +2061,7 @@
         <v>60</v>
       </c>
       <c r="J2" s="3" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3">
@@ -2103,7 +2103,7 @@
         <v>52</v>
       </c>
       <c r="J3" s="3" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="4">
@@ -2145,7 +2145,7 @@
         <v>60</v>
       </c>
       <c r="J4" s="3" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5">
@@ -2187,7 +2187,7 @@
         <v>60</v>
       </c>
       <c r="J5" s="3" t="n">
-        <v>0</v>
+        <v>-2</v>
       </c>
     </row>
     <row r="6">
@@ -2229,7 +2229,7 @@
         <v>60</v>
       </c>
       <c r="J6" s="3" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7">
@@ -2271,7 +2271,7 @@
         <v>60</v>
       </c>
       <c r="J7" s="3" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="8">
@@ -2313,7 +2313,7 @@
         <v>60</v>
       </c>
       <c r="J8" s="3" t="n">
-        <v>0</v>
+        <v>-2</v>
       </c>
     </row>
     <row r="9">
@@ -2355,7 +2355,7 @@
         <v>52</v>
       </c>
       <c r="J9" s="3" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="10">
@@ -2397,7 +2397,7 @@
         <v>66</v>
       </c>
       <c r="J10" s="3" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="11">
@@ -2439,7 +2439,7 @@
         <v>75</v>
       </c>
       <c r="J11" s="3" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -2558,7 +2558,7 @@
         <v>67</v>
       </c>
       <c r="J2" s="3" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3">
@@ -2600,7 +2600,7 @@
         <v>135</v>
       </c>
       <c r="J3" s="3" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4">
@@ -2642,7 +2642,7 @@
         <v>150</v>
       </c>
       <c r="J4" s="3" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="5">
@@ -2684,7 +2684,7 @@
         <v>45</v>
       </c>
       <c r="J5" s="3" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="6">
@@ -2726,7 +2726,7 @@
         <v>180</v>
       </c>
       <c r="J6" s="3" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7">
@@ -2768,7 +2768,7 @@
         <v>120</v>
       </c>
       <c r="J7" s="3" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="8">
@@ -2810,7 +2810,7 @@
         <v>75</v>
       </c>
       <c r="J8" s="3" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9">
@@ -2852,7 +2852,7 @@
         <v>120</v>
       </c>
       <c r="J9" s="3" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10">
@@ -2894,7 +2894,7 @@
         <v>135</v>
       </c>
       <c r="J10" s="3" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="11">
@@ -2936,7 +2936,7 @@
         <v>165</v>
       </c>
       <c r="J11" s="3" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -3055,7 +3055,7 @@
         <v>195</v>
       </c>
       <c r="J2" s="3" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3">
@@ -3097,7 +3097,7 @@
         <v>150</v>
       </c>
       <c r="J3" s="3" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4">
@@ -3139,7 +3139,7 @@
         <v>105</v>
       </c>
       <c r="J4" s="3" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="5">
@@ -3181,7 +3181,7 @@
         <v>150</v>
       </c>
       <c r="J5" s="3" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6">
@@ -3223,7 +3223,7 @@
         <v>210</v>
       </c>
       <c r="J6" s="3" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7">
@@ -3265,7 +3265,7 @@
         <v>120</v>
       </c>
       <c r="J7" s="3" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="8">
@@ -3307,7 +3307,7 @@
         <v>120</v>
       </c>
       <c r="J8" s="3" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="9">
@@ -3349,7 +3349,7 @@
         <v>135</v>
       </c>
       <c r="J9" s="3" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10">
@@ -3391,7 +3391,7 @@
         <v>165</v>
       </c>
       <c r="J10" s="3" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="11">
@@ -3433,7 +3433,7 @@
         <v>120</v>
       </c>
       <c r="J11" s="3" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -3553,7 +3553,7 @@
         <v>97</v>
       </c>
       <c r="J2" s="3" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="3">
@@ -3595,7 +3595,7 @@
         <v>58</v>
       </c>
       <c r="J3" s="3" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4">
@@ -3637,7 +3637,7 @@
         <v>240</v>
       </c>
       <c r="J4" s="3" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -3679,7 +3679,7 @@
         <v>105</v>
       </c>
       <c r="J5" s="3" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="6">
@@ -3721,7 +3721,7 @@
         <v>150</v>
       </c>
       <c r="J6" s="3" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="7">
@@ -3763,7 +3763,7 @@
         <v>90</v>
       </c>
       <c r="J7" s="3" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8">
@@ -3805,7 +3805,7 @@
         <v>96</v>
       </c>
       <c r="J8" s="3" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9">
@@ -3847,7 +3847,7 @@
         <v>120</v>
       </c>
       <c r="J9" s="3" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="10">
@@ -3889,7 +3889,7 @@
         <v>120</v>
       </c>
       <c r="J10" s="3" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="11">
@@ -3931,7 +3931,7 @@
         <v>135</v>
       </c>
       <c r="J11" s="3" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -4050,7 +4050,7 @@
         <v>178</v>
       </c>
       <c r="J2" s="3" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="3">
@@ -4092,7 +4092,7 @@
         <v>93</v>
       </c>
       <c r="J3" s="3" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="4">
@@ -4134,7 +4134,7 @@
         <v>150</v>
       </c>
       <c r="J4" s="3" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="5">
@@ -4176,7 +4176,7 @@
         <v>217</v>
       </c>
       <c r="J5" s="3" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="6">
@@ -4218,7 +4218,7 @@
         <v>99</v>
       </c>
       <c r="J6" s="3" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="7">
@@ -4260,7 +4260,7 @@
         <v>150</v>
       </c>
       <c r="J7" s="3" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="8">
@@ -4302,7 +4302,7 @@
         <v>135</v>
       </c>
       <c r="J8" s="3" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="9">
@@ -4344,7 +4344,7 @@
         <v>120</v>
       </c>
       <c r="J9" s="3" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="10">
@@ -4386,7 +4386,7 @@
         <v>90</v>
       </c>
       <c r="J10" s="3" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="11">
@@ -4428,7 +4428,7 @@
         <v>165</v>
       </c>
       <c r="J11" s="3" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -4547,7 +4547,7 @@
         <v>37</v>
       </c>
       <c r="J2" s="3" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="3">
@@ -4589,7 +4589,7 @@
         <v>45</v>
       </c>
       <c r="J3" s="3" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4">
@@ -4631,7 +4631,7 @@
         <v>90</v>
       </c>
       <c r="J4" s="3" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5">
@@ -4673,7 +4673,7 @@
         <v>33</v>
       </c>
       <c r="J5" s="3" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="6">
@@ -4715,7 +4715,7 @@
         <v>52</v>
       </c>
       <c r="J6" s="3" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="7">
@@ -4757,7 +4757,7 @@
         <v>42</v>
       </c>
       <c r="J7" s="3" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="8">
@@ -4799,7 +4799,7 @@
         <v>60</v>
       </c>
       <c r="J8" s="3" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="9">
@@ -4841,7 +4841,7 @@
         <v>150</v>
       </c>
       <c r="J9" s="3" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10">
@@ -4883,7 +4883,7 @@
         <v>66</v>
       </c>
       <c r="J10" s="3" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="11">
@@ -4925,7 +4925,7 @@
         <v>37</v>
       </c>
       <c r="J11" s="3" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -5045,7 +5045,7 @@
         <v>120</v>
       </c>
       <c r="J2" s="3" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3">
@@ -5087,7 +5087,7 @@
         <v>57</v>
       </c>
       <c r="J3" s="3" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4">
@@ -5129,7 +5129,7 @@
         <v>114</v>
       </c>
       <c r="J4" s="3" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="5">
@@ -5171,7 +5171,7 @@
         <v>165</v>
       </c>
       <c r="J5" s="3" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6">
@@ -5213,7 +5213,7 @@
         <v>135</v>
       </c>
       <c r="J6" s="3" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7">
@@ -5255,7 +5255,7 @@
         <v>150</v>
       </c>
       <c r="J7" s="3" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8">
@@ -5297,7 +5297,7 @@
         <v>105</v>
       </c>
       <c r="J8" s="3" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="9">
@@ -5339,7 +5339,7 @@
         <v>150</v>
       </c>
       <c r="J9" s="3" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10">
@@ -5381,7 +5381,7 @@
         <v>135</v>
       </c>
       <c r="J10" s="3" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="11">
@@ -5423,7 +5423,7 @@
         <v>120</v>
       </c>
       <c r="J11" s="3" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>